<commit_message>
fix: clear stale REPORT styling and give the payment panel its own picker
The payment REPORT sheet is built on top of the monthly report's "REPORT 2"
sheet, whose layout differs. Clearing only the values left its fills and
borders behind, so empty spacer cells (C3, row 5, C6, C7) rendered as stray
orange and blue bands. Reset each cell's style as well as its value.

The Reports page's payment panel now carries its own VALD / Bodydot picker
instead of following the report side's Service toggle, and uses flex gap
rather than space-y so its lg:hidden heading stops pushing the picker out
of line with the one opposite it.

Blob error bodies are now read back as text, so a failed payment request
shows the server's detail instead of failing silently — this affected the
VALD payment report too.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bodydot Payment - Month YEAR.xlsx
+++ b/Bodydot Payment - Month YEAR.xlsx
@@ -774,21 +774,9 @@
         </is>
       </c>
       <c r="B3" s="23" t="n"/>
-      <c r="C3" s="43" t="n"/>
-      <c r="D3" s="15" t="n"/>
-    </row>
-    <row r="4" ht="47.75" customHeight="1">
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="26" t="n"/>
-      <c r="D4" s="1" t="n"/>
-    </row>
-    <row r="5" ht="47.75" customHeight="1">
-      <c r="A5" s="38" t="n"/>
-      <c r="B5" s="38" t="n"/>
-      <c r="C5" s="39" t="n"/>
-      <c r="D5" s="40" t="n"/>
-      <c r="F5" s="5" t="n"/>
-    </row>
+    </row>
+    <row r="4" ht="47.75" customHeight="1"/>
+    <row r="5" ht="47.75" customHeight="1"/>
     <row r="6" ht="49.25" customHeight="1">
       <c r="A6" s="56" t="inlineStr">
         <is>
@@ -796,14 +784,12 @@
         </is>
       </c>
       <c r="B6" s="38" t="n"/>
-      <c r="C6" s="42" t="n"/>
       <c r="D6" s="56" t="inlineStr">
         <is>
           <t>BODY MOTIONS BRANCHES</t>
         </is>
       </c>
       <c r="E6" s="38" t="n"/>
-      <c r="F6" s="5" t="n"/>
       <c r="G6" s="57" t="inlineStr">
         <is>
           <t>TOTAL GYMS</t>
@@ -823,7 +809,6 @@
           <t>Total Tests</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n"/>
       <c r="D7" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">CLUB NAME
@@ -859,7 +844,6 @@
           <t>إجمالي الاختبارات</t>
         </is>
       </c>
-      <c r="C8" s="11" t="n"/>
       <c r="D8" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">اسم النادي
@@ -890,7 +874,6 @@
         </is>
       </c>
       <c r="B9" s="21" t="n"/>
-      <c r="C9" s="11" t="n"/>
       <c r="D9" s="25" t="inlineStr">
         <is>
           <t>RUH - Al Sahafa</t>
@@ -908,11 +891,6 @@
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="10" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="10" t="n"/>
       <c r="G10" s="25" t="inlineStr">
         <is>
           <t>Body Masters</t>
@@ -923,272 +901,44 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="10" t="n"/>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="10" t="n"/>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="10" t="n"/>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="10" t="n"/>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="10" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="10" t="n"/>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="10" t="n"/>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="10" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="10" t="n"/>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="10" t="n"/>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="10" t="n"/>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="10" t="n"/>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="10" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="10" t="n"/>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="10" t="n"/>
-      <c r="B21" s="10" t="n"/>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
-      <c r="E21" s="10" t="n"/>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="10" t="n"/>
-      <c r="B22" s="10" t="n"/>
-      <c r="C22" s="11" t="n"/>
-      <c r="D22" s="11" t="n"/>
-      <c r="E22" s="10" t="n"/>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="10" t="n"/>
-      <c r="B23" s="10" t="n"/>
-      <c r="C23" s="11" t="n"/>
-      <c r="D23" s="11" t="n"/>
-      <c r="E23" s="10" t="n"/>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="10" t="n"/>
-      <c r="B24" s="10" t="n"/>
-      <c r="C24" s="11" t="n"/>
-      <c r="D24" s="11" t="n"/>
-      <c r="E24" s="10" t="n"/>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="10" t="n"/>
-      <c r="B25" s="10" t="n"/>
-      <c r="C25" s="11" t="n"/>
-      <c r="D25" s="11" t="n"/>
-      <c r="E25" s="10" t="n"/>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="10" t="n"/>
-      <c r="B26" s="10" t="n"/>
-      <c r="C26" s="11" t="n"/>
-      <c r="D26" s="11" t="n"/>
-      <c r="E26" s="10" t="n"/>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="10" t="n"/>
-      <c r="B27" s="10" t="n"/>
-      <c r="C27" s="11" t="n"/>
-      <c r="D27" s="11" t="n"/>
-      <c r="E27" s="10" t="n"/>
-    </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="10" t="n"/>
-      <c r="B28" s="10" t="n"/>
-      <c r="C28" s="11" t="n"/>
-      <c r="D28" s="11" t="n"/>
-      <c r="E28" s="10" t="n"/>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="10" t="n"/>
-      <c r="B29" s="10" t="n"/>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="11" t="n"/>
-      <c r="E29" s="10" t="n"/>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="10" t="n"/>
-      <c r="B30" s="10" t="n"/>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="11" t="n"/>
-      <c r="E30" s="10" t="n"/>
-    </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="10" t="n"/>
-      <c r="B31" s="10" t="n"/>
-      <c r="C31" s="11" t="n"/>
-      <c r="D31" s="11" t="n"/>
-      <c r="E31" s="10" t="n"/>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="10" t="n"/>
-      <c r="B32" s="10" t="n"/>
-      <c r="C32" s="11" t="n"/>
-      <c r="D32" s="11" t="n"/>
-      <c r="E32" s="10" t="n"/>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="10" t="n"/>
-      <c r="B33" s="10" t="n"/>
-      <c r="C33" s="11" t="n"/>
-      <c r="D33" s="11" t="n"/>
-      <c r="E33" s="10" t="n"/>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="10" t="n"/>
-      <c r="B34" s="10" t="n"/>
-      <c r="C34" s="11" t="n"/>
-      <c r="D34" s="11" t="n"/>
-      <c r="E34" s="10" t="n"/>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="10" t="n"/>
-      <c r="B35" s="10" t="n"/>
-      <c r="C35" s="11" t="n"/>
-      <c r="D35" s="11" t="n"/>
-      <c r="E35" s="10" t="n"/>
-    </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="10" t="n"/>
-      <c r="B36" s="10" t="n"/>
-      <c r="C36" s="11" t="n"/>
-      <c r="D36" s="11" t="n"/>
-      <c r="E36" s="10" t="n"/>
-    </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="10" t="n"/>
-      <c r="B37" s="10" t="n"/>
-      <c r="C37" s="11" t="n"/>
-      <c r="D37" s="11" t="n"/>
-      <c r="E37" s="10" t="n"/>
-    </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="10" t="n"/>
-      <c r="B38" s="10" t="n"/>
-      <c r="C38" s="11" t="n"/>
-      <c r="D38" s="11" t="n"/>
-      <c r="E38" s="10" t="n"/>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="10" t="n"/>
-      <c r="B39" s="10" t="n"/>
-      <c r="C39" s="11" t="n"/>
-      <c r="D39" s="11" t="n"/>
-      <c r="E39" s="10" t="n"/>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="10" t="n"/>
-      <c r="B40" s="10" t="n"/>
-      <c r="C40" s="11" t="n"/>
-      <c r="D40" s="11" t="n"/>
-      <c r="E40" s="10" t="n"/>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="10" t="n"/>
-      <c r="B41" s="10" t="n"/>
-      <c r="C41" s="11" t="n"/>
-      <c r="D41" s="11" t="n"/>
-      <c r="E41" s="10" t="n"/>
-    </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="10" t="n"/>
-      <c r="B42" s="10" t="n"/>
-      <c r="C42" s="11" t="n"/>
-      <c r="D42" s="11" t="n"/>
-      <c r="E42" s="10" t="n"/>
-    </row>
-    <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="10" t="n"/>
-      <c r="B43" s="10" t="n"/>
-      <c r="C43" s="11" t="n"/>
-      <c r="D43" s="11" t="n"/>
-      <c r="E43" s="10" t="n"/>
-    </row>
-    <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="10" t="n"/>
-      <c r="B44" s="10" t="n"/>
-      <c r="C44" s="11" t="n"/>
-      <c r="D44" s="11" t="n"/>
-      <c r="E44" s="10" t="n"/>
-    </row>
-    <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="10" t="n"/>
-      <c r="B45" s="10" t="n"/>
-      <c r="C45" s="11" t="n"/>
-      <c r="D45" s="11" t="n"/>
-      <c r="E45" s="10" t="n"/>
-    </row>
-    <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="10" t="n"/>
-      <c r="B46" s="10" t="n"/>
-      <c r="C46" s="11" t="n"/>
-      <c r="D46" s="11" t="n"/>
-      <c r="E46" s="10" t="n"/>
-    </row>
-    <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="10" t="n"/>
-      <c r="B47" s="10" t="n"/>
-      <c r="C47" s="11" t="n"/>
-      <c r="D47" s="11" t="n"/>
-      <c r="E47" s="10" t="n"/>
-    </row>
-    <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="10" t="n"/>
-      <c r="B48" s="10" t="n"/>
-      <c r="C48" s="11" t="n"/>
-      <c r="D48" s="11" t="n"/>
-      <c r="E48" s="10" t="n"/>
-    </row>
+    <row r="11" ht="16" customHeight="1"/>
+    <row r="12" ht="16" customHeight="1"/>
+    <row r="13" ht="16" customHeight="1"/>
+    <row r="14" ht="16" customHeight="1"/>
+    <row r="15" ht="16" customHeight="1"/>
+    <row r="16" ht="16" customHeight="1"/>
+    <row r="17" ht="16" customHeight="1"/>
+    <row r="18" ht="16" customHeight="1"/>
+    <row r="19" ht="16" customHeight="1"/>
+    <row r="20" ht="16" customHeight="1"/>
+    <row r="21" ht="16" customHeight="1"/>
+    <row r="22" ht="16" customHeight="1"/>
+    <row r="23" ht="16" customHeight="1"/>
+    <row r="24" ht="16" customHeight="1"/>
+    <row r="25" ht="16" customHeight="1"/>
+    <row r="26" ht="16" customHeight="1"/>
+    <row r="27" ht="16" customHeight="1"/>
+    <row r="28" ht="16" customHeight="1"/>
+    <row r="29" ht="16" customHeight="1"/>
+    <row r="30" ht="16" customHeight="1"/>
+    <row r="31" ht="16" customHeight="1"/>
+    <row r="32" ht="16" customHeight="1"/>
+    <row r="33" ht="16" customHeight="1"/>
+    <row r="34" ht="16" customHeight="1"/>
+    <row r="35" ht="16" customHeight="1"/>
+    <row r="36" ht="16" customHeight="1"/>
+    <row r="37" ht="16" customHeight="1"/>
+    <row r="38" ht="16" customHeight="1"/>
+    <row r="39" ht="16" customHeight="1"/>
+    <row r="40" ht="16" customHeight="1"/>
+    <row r="41" ht="16" customHeight="1"/>
+    <row r="42" ht="16" customHeight="1"/>
+    <row r="43" ht="16" customHeight="1"/>
+    <row r="44" ht="16" customHeight="1"/>
+    <row r="45" ht="16" customHeight="1"/>
+    <row r="46" ht="16" customHeight="1"/>
+    <row r="47" ht="16" customHeight="1"/>
+    <row r="48" ht="16" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="D6:E6"/>

</xml_diff>

<commit_message>
fix: carry sheet view and print setup onto the copied Motions sheet
wb.copy_worksheet() duplicates cells and styles but not the sheet view or
header/footer, so "Body Motions - RUH - Al Sahafa" opened at 100% zoom with
gridlines showing while every other sheet sat at 50% with them off. Copy the
views and header across after the duplication.

Print areas are now sized to the rows actually written instead of inheriting
the report template's 16-row area, which would have cut printing short on a
sheet that regularly runs past 70 rows.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bodydot Payment - Month YEAR.xlsx
+++ b/Bodydot Payment - Month YEAR.xlsx
@@ -12,8 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'REPORT'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'REPORT'!$A$1:$G$7</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Body Masters - RUH - Al Aarid'!$B$1:$H$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'REPORT'!$A$1:$H$10</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -2624,6 +2623,14 @@
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" scale="41"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;G</oddHeader>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 

</xml_diff>